<commit_message>
Add 9 tests to the Test Plan Matrix
</commit_message>
<xml_diff>
--- a/Iteration 3/Test Plan Matrix.xlsx
+++ b/Iteration 3/Test Plan Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sara\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://temahau-my.sharepoint.com/personal/scatta1_student_eit_ac_nz/Documents/Desktop/AgileProject/AgileProjects_Repository/Iteration 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{398062F4-2FAF-4125-AEB4-BD443E83F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="100" documentId="13_ncr:1_{398062F4-2FAF-4125-AEB4-BD443E83F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10AFD676-1C70-4929-88C4-6F20F7A90295}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{DD13817E-CF7B-49AF-9A2F-4CD4F0533F38}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD13817E-CF7B-49AF-9A2F-4CD4F0533F38}"/>
   </bookViews>
   <sheets>
     <sheet name="UAT" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>User Acceptance Test Plan</t>
   </si>
@@ -96,13 +96,142 @@
   </si>
   <si>
     <t>ORDERS PAGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Reponse Time </t>
+  </si>
+  <si>
+    <t>Open Developer Tools, open networking, refresh page</t>
+  </si>
+  <si>
+    <t>Page fully loads with all content within 2-3 Secounds</t>
+  </si>
+  <si>
+    <t>Pages contents loaded in 1.52 seconds</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t>Hover animation on the "Features Of Our Watches" section</t>
+  </si>
+  <si>
+    <t>navigate to the features section, Hover curser on the fitness tracking, alerts and notifications, messages and bluetooth boxes</t>
+  </si>
+  <si>
+    <t>All Hover animations activate when the curser is above the the box</t>
+  </si>
+  <si>
+    <t>All boxes had a successful hover animation when curser was hovering them</t>
+  </si>
+  <si>
+    <t>Testimonial foward carousel button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">navigate to the testimonial section, click both the left and right arrow buttons displayed under the carousel </t>
+  </si>
+  <si>
+    <t>Once the left or right arrow button is clicked the above box will display an animation to change the box to next or previous box.</t>
+  </si>
+  <si>
+    <t>Once clicked the left arrow button changed the box to the prevoius box with an animation. The right arrow butto when clicked changed the box to the next box in the carousel</t>
+  </si>
+  <si>
+    <t>Test the Phone display changes to the correct display proportions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open Develpper tools and change the page display to the phone option and navigate the page </t>
+  </si>
+  <si>
+    <t>Page successfully changes proportions to accoudate the display</t>
+  </si>
+  <si>
+    <t>Contact Us button redirects to the contacts page</t>
+  </si>
+  <si>
+    <t>Page displayed as phone and successfully accommodated the display by changing proportions</t>
+  </si>
+  <si>
+    <t>Click the Contact us button on the Slider Section card</t>
+  </si>
+  <si>
+    <t>On clicking the button the page should redirect the user to a contacts page</t>
+  </si>
+  <si>
+    <t>On clicking the button the page didn’t redirect but instead refreshed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fail </t>
+  </si>
+  <si>
+    <t>Each Product card when clicked displays the product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click each product card link </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Product card link will open a page on the product with details </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Product cards when clicked redirected to the watches page rather than the watch details </t>
+  </si>
+  <si>
+    <t>fail</t>
+  </si>
+  <si>
+    <t>Header Links on watches page redirect the user to the linked page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click on each link displayed on the header </t>
+  </si>
+  <si>
+    <t>The Header links redirect the user to the page listed</t>
+  </si>
+  <si>
+    <t>Each link when clicked redircts you to the page it listed as a link</t>
+  </si>
+  <si>
+    <t>View all Button clicked changes the viewing display of the products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click on the View All link under all the products </t>
+  </si>
+  <si>
+    <t xml:space="preserve">the View All button will change the layout and display of the product cards listed </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The View all button when clicked redirts you to the watches page without changing the layout of the product cards </t>
+  </si>
+  <si>
+    <t>The Cart Button when clicked reloads the current page</t>
+  </si>
+  <si>
+    <t>Click the Cart Icon Button in the top right corner of the header</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Cart Button redirects the user to the Cart page </t>
+  </si>
+  <si>
+    <t>The Product cards redirect the user to the watches page instead of</t>
+  </si>
+  <si>
+    <t>The View All button Refreshes the watches page instead of changing the layout or redirecting the user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cart Icon Button takes the user to the cart page </t>
+  </si>
+  <si>
+    <t>Cart Button Reloads the page the user is currently on instead of redirecting to the Cart page.</t>
+  </si>
+  <si>
+    <t>Button redircets the user to the home page rather than the contacts page</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -229,6 +358,24 @@
       <b/>
       <sz val="18"/>
       <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7.5"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -490,7 +637,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -550,50 +697,32 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -615,6 +744,12 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -627,11 +762,41 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -950,42 +1115,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DE0EC2B-16AC-4837-9A90-74B674A1A8AC}">
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.54296875" customWidth="1"/>
-    <col min="2" max="2" width="28.26953125" customWidth="1"/>
-    <col min="3" max="3" width="26.54296875" customWidth="1"/>
-    <col min="4" max="4" width="32.26953125" customWidth="1"/>
-    <col min="5" max="5" width="27.7265625" customWidth="1"/>
-    <col min="6" max="6" width="49.1796875" customWidth="1"/>
-    <col min="7" max="7" width="37.7265625" customWidth="1"/>
-    <col min="9" max="9" width="13.1796875" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" customWidth="1"/>
+    <col min="1" max="1" width="6.5703125" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" customWidth="1"/>
+    <col min="5" max="5" width="27.7109375" customWidth="1"/>
+    <col min="6" max="6" width="49.140625" customWidth="1"/>
+    <col min="7" max="7" width="37.7109375" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31" x14ac:dyDescent="0.7">
-      <c r="A1" s="40"/>
-      <c r="B1" s="41"/>
-      <c r="C1" s="38" t="s">
+    <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
+      <c r="A1" s="34"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="44" t="s">
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="49" t="s">
+      <c r="B2" s="39"/>
+      <c r="C2" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="49"/>
+      <c r="D2" s="45"/>
       <c r="E2" s="11"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -993,11 +1158,11 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="50" t="s">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="51"/>
+      <c r="B3" s="41"/>
       <c r="C3" s="19" t="s">
         <v>14</v>
       </c>
@@ -1009,15 +1174,15 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="46" t="s">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="47"/>
-      <c r="C4" s="21" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="22"/>
+      <c r="D4" s="49"/>
       <c r="E4" s="11"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1025,29 +1190,29 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="48"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-    </row>
-    <row r="6" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="44"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="C6" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="24"/>
+      <c r="D6" s="51"/>
       <c r="E6" s="12" t="s">
         <v>6</v>
       </c>
@@ -1060,180 +1225,278 @@
       <c r="H6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="42" t="s">
+      <c r="I6" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="43"/>
-    </row>
-    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="J6" s="37"/>
+    </row>
+    <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="7"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="37"/>
-    </row>
-    <row r="8" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="28"/>
+    </row>
+    <row r="8" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>1</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="26"/>
+      <c r="B8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="47"/>
       <c r="E8" s="18"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="35"/>
-    </row>
-    <row r="9" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="F8" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="52"/>
+      <c r="J8" s="24"/>
+    </row>
+    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>2</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="26"/>
+      <c r="B9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="47"/>
       <c r="E9" s="3"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
-    </row>
-    <row r="10" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="F9" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="23"/>
+      <c r="J9" s="24"/>
+    </row>
+    <row r="10" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>3</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26"/>
+      <c r="B10" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="47"/>
       <c r="E10" s="3"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="17"/>
+      <c r="F10" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G10" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="17" t="s">
+        <v>24</v>
+      </c>
       <c r="I10" s="4"/>
       <c r="J10" s="5"/>
     </row>
-    <row r="11" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>4</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="26"/>
+      <c r="B11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="54"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="35"/>
-    </row>
-    <row r="12" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="13" t="s">
+      <c r="F11" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I11" s="4"/>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="47"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" s="55" t="s">
+        <v>62</v>
+      </c>
+      <c r="J12" s="24"/>
+    </row>
+    <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="37"/>
-    </row>
-    <row r="13" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="2">
+      <c r="B13" s="14"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="28"/>
+    </row>
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
         <v>1</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="35"/>
-    </row>
-    <row r="14" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="2">
+      <c r="B14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="30"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="J14" s="24"/>
+    </row>
+    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>2</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="35"/>
-    </row>
-    <row r="15" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="2">
+      <c r="B15" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="22"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+    </row>
+    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
         <v>3</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="33"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="35"/>
-    </row>
-    <row r="16" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="2">
+      <c r="B16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D16" s="22"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="J16" s="24"/>
+    </row>
+    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
         <v>4</v>
       </c>
-      <c r="B16" s="3"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="5"/>
-    </row>
-    <row r="17" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="2">
-        <v>5</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="28"/>
+      <c r="B17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" s="22"/>
       <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="35"/>
-    </row>
-    <row r="18" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="F17" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="J17" s="57"/>
+    </row>
+    <row r="18" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B18" s="14"/>
-      <c r="C18" s="36"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="36"/>
-      <c r="J18" s="37"/>
-    </row>
-    <row r="19" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="28"/>
+    </row>
+    <row r="19" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>1</v>
       </c>
@@ -1244,44 +1507,44 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="17"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="35"/>
-    </row>
-    <row r="20" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I19" s="23"/>
+      <c r="J19" s="24"/>
+    </row>
+    <row r="20" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>2</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
+      <c r="D20" s="22"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="15"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="35"/>
-    </row>
-    <row r="21" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I20" s="23"/>
+      <c r="J20" s="24"/>
+    </row>
+    <row r="21" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>3</v>
       </c>
       <c r="B21" s="3"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="32"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="15"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="35"/>
-    </row>
-    <row r="22" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I21" s="23"/>
+      <c r="J21" s="24"/>
+    </row>
+    <row r="22" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>4</v>
       </c>
       <c r="B22" s="3"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="32"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="22"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1289,35 +1552,35 @@
       <c r="I22" s="4"/>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>5</v>
       </c>
       <c r="B23" s="3"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="28"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="26"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="15"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="35"/>
-    </row>
-    <row r="24" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="I23" s="23"/>
+      <c r="J23" s="24"/>
+    </row>
+    <row r="24" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="14"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="36"/>
-      <c r="J24" s="37"/>
-    </row>
-    <row r="25" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="28"/>
+    </row>
+    <row r="25" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>1</v>
       </c>
@@ -1328,44 +1591,44 @@
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="17"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="35"/>
-    </row>
-    <row r="26" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I25" s="23"/>
+      <c r="J25" s="24"/>
+    </row>
+    <row r="26" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>2</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
+      <c r="D26" s="22"/>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="15"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="35"/>
-    </row>
-    <row r="27" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I26" s="23"/>
+      <c r="J26" s="24"/>
+    </row>
+    <row r="27" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>3</v>
       </c>
       <c r="B27" s="3"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="32"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="15"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="35"/>
-    </row>
-    <row r="28" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I27" s="23"/>
+      <c r="J27" s="24"/>
+    </row>
+    <row r="28" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>4</v>
       </c>
       <c r="B28" s="3"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="32"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -1373,35 +1636,35 @@
       <c r="I28" s="4"/>
       <c r="J28" s="5"/>
     </row>
-    <row r="29" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>5</v>
       </c>
       <c r="B29" s="3"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="28"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="26"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="15"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="35"/>
-    </row>
-    <row r="30" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="I29" s="23"/>
+      <c r="J29" s="24"/>
+    </row>
+    <row r="30" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B30" s="14"/>
-      <c r="C30" s="36"/>
-      <c r="D30" s="36"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="36"/>
-      <c r="J30" s="37"/>
-    </row>
-    <row r="31" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="27"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="28"/>
+    </row>
+    <row r="31" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>1</v>
       </c>
@@ -1412,44 +1675,44 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="17"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="35"/>
-    </row>
-    <row r="32" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I31" s="23"/>
+      <c r="J31" s="24"/>
+    </row>
+    <row r="32" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>2</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="31"/>
-      <c r="D32" s="32"/>
+      <c r="D32" s="22"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="15"/>
-      <c r="I32" s="34"/>
-      <c r="J32" s="35"/>
-    </row>
-    <row r="33" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I32" s="23"/>
+      <c r="J32" s="24"/>
+    </row>
+    <row r="33" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>3</v>
       </c>
       <c r="B33" s="3"/>
-      <c r="C33" s="33"/>
-      <c r="D33" s="32"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="22"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="H33" s="15"/>
-      <c r="I33" s="34"/>
-      <c r="J33" s="35"/>
-    </row>
-    <row r="34" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="I33" s="23"/>
+      <c r="J33" s="24"/>
+    </row>
+    <row r="34" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>4</v>
       </c>
       <c r="B34" s="3"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="32"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="22"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -1457,80 +1720,80 @@
       <c r="I34" s="4"/>
       <c r="J34" s="5"/>
     </row>
-    <row r="35" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>5</v>
       </c>
       <c r="B35" s="3"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="28"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="26"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="H35" s="15"/>
-      <c r="I35" s="34"/>
-      <c r="J35" s="35"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C18:J18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="C1:J1"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I14:J14"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="C24:J24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="C30:J30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="I32:J32"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="I33:J33"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="C35:D35"/>
     <mergeCell ref="I35:J35"/>
-    <mergeCell ref="C30:J30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C24:J24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="C1:J1"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="I17:J17"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C12:J12"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="C18:J18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
added testing results for site contact & footer
</commit_message>
<xml_diff>
--- a/Iteration 3/Test Plan Matrix.xlsx
+++ b/Iteration 3/Test Plan Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://temahau-my.sharepoint.com/personal/scatta1_student_eit_ac_nz/Documents/Desktop/AgileProject/AgileProjects_Repository/Iteration 3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://temahau-my.sharepoint.com/personal/sellws2_student_eit_ac_nz/Documents/Documents/ITPM5.240 Agile Projects/Assignments/AgileProjects_Repository/Iteration 3/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="100" documentId="13_ncr:1_{398062F4-2FAF-4125-AEB4-BD443E83F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10AFD676-1C70-4929-88C4-6F20F7A90295}"/>
+  <xr:revisionPtr revIDLastSave="187" documentId="13_ncr:1_{398062F4-2FAF-4125-AEB4-BD443E83F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0F808C9-C840-4C54-B472-8CF3F7D67E79}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD13817E-CF7B-49AF-9A2F-4CD4F0533F38}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{DD13817E-CF7B-49AF-9A2F-4CD4F0533F38}"/>
   </bookViews>
   <sheets>
     <sheet name="UAT" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="97">
   <si>
     <t>User Acceptance Test Plan</t>
   </si>
@@ -225,6 +225,108 @@
   </si>
   <si>
     <t>Button redircets the user to the home page rather than the contacts page</t>
+  </si>
+  <si>
+    <t>Inputting text into the contact us form and submitting</t>
+  </si>
+  <si>
+    <t>Simply adding text to the name fields, email field and message field and seeing what happens.</t>
+  </si>
+  <si>
+    <t>Notification saying "Sent" to confirm the message has been sent. Error message if sending failed and inform user reason why. Should not be able to input alphabetic characters for phone number. Error notification for invalid inputs e.g. invalid/incomplete email address, phone number.</t>
+  </si>
+  <si>
+    <t>When pressing send page refreshes, doesn't send. Able to input text in every field - even phone number. Error notification for not having an "@" in email - will show "Please enter an email address". No "sent" confirmation.</t>
+  </si>
+  <si>
+    <t>Lacks to inform user of errors or confirmations, contact form message is not being sent.</t>
+  </si>
+  <si>
+    <t>Clicking header menu links from Contact Us page</t>
+  </si>
+  <si>
+    <t>Clicking on each page link to test if the links are redirecting the user to the correct page.</t>
+  </si>
+  <si>
+    <t>"sara" in each field, adding "@" in email field and ".com"</t>
+  </si>
+  <si>
+    <t>Each link redirecting to correct page e.g. clicking "Home" and being redirected to the Home page, clicking "Watches" and being redirected to the Watches collection page, etc. User cursor "hand" displayed over link hover.</t>
+  </si>
+  <si>
+    <t>Each link was clicked starting from the Contact Us page for each one and redirected to the associated page. Cursor showed a hand over every link to inform user that the link was interactive when clicked.</t>
+  </si>
+  <si>
+    <t>Passed but could add a hover over colour to also help user identify that it is a working interactive link and the cursor is hovering the link.</t>
+  </si>
+  <si>
+    <t>FOOTERS/HEADERS</t>
+  </si>
+  <si>
+    <t>Adding text into the email field and pressing the subscribe button.</t>
+  </si>
+  <si>
+    <t>Notification saying "Subscribed" to confirm the subscription has been successful. Error message if sending failed and inform user reason why e.g. invalid email or characters.</t>
+  </si>
+  <si>
+    <t>Subscription form not set up correctly, doesn't submit email address, just refreshes the page.</t>
+  </si>
+  <si>
+    <t>Clicking header menu links from all menu pages</t>
+  </si>
+  <si>
+    <t>Google Map located bottom right at footer</t>
+  </si>
+  <si>
+    <t>"Subscribe" form located at footer on every page of website</t>
+  </si>
+  <si>
+    <t>Fullscreening, pressing "ok" on notification and navigating the map.</t>
+  </si>
+  <si>
+    <t>Map should show the location of the Timups Store for users to locate in case they want to visit the physical store.</t>
+  </si>
+  <si>
+    <t>Map shows message "This page can't load Google Maps correctly" and pressing "ok" doesn't update the page. By default it is displaying New York City and shows a watermark saying "for development purposes only".</t>
+  </si>
+  <si>
+    <t>Not showing correct location/not working. Need to fix widget to show correct location of store.</t>
+  </si>
+  <si>
+    <t>Locate link to privacy information, detailing how the website collects user information upon visiting the website.</t>
+  </si>
+  <si>
+    <t>No privacy link in the footer.</t>
+  </si>
+  <si>
+    <t>Observation, navigating links in the footer area.</t>
+  </si>
+  <si>
+    <t>Website needs a privacy statement for compliance (Web Usability Standard).</t>
+  </si>
+  <si>
+    <t>Missing Terms &amp; Conditions, Privacy statement links</t>
+  </si>
+  <si>
+    <t>When pressing subscribe the page refreshes. No text entered and pressed "subscribe" still refreshes - no errors. No limited on how many characters can be inputted.</t>
+  </si>
+  <si>
+    <t>Footer contact links, email, phone, social media links and login icons in header</t>
+  </si>
+  <si>
+    <t>Clicking on each link to see if it redirects the user to the associated label e.g. sending an email or directed to instagram clicking on logo image. Clicking on login icons in top right to see outcome.</t>
+  </si>
+  <si>
+    <t>Each link redirecting user to the correct place, all social media links to respective site profile. Opening email (e.g. Outlook) to send an email, after clicking on email address. Asking user to conform call when clicking on phone number. Login icons should let you sign in/sign up, view account information including card info, purchase history and accouting settings. As well as shopping cart details and being able to click the magnifying icon to search the site.</t>
+  </si>
+  <si>
+    <t>All links, social media icons and login icons would refresh the page. This was the outcome for each page.</t>
+  </si>
+  <si>
+    <t>All links and icons refreshing page/incorrect links - not working how expected to. Unable to login / sign up to the website or add to cart / purchase items.</t>
+  </si>
+  <si>
+    <t>"sara" in email field and spamming alphanumerical characters to test character limit</t>
   </si>
 </sst>
 </file>
@@ -637,7 +739,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -697,20 +799,45 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -718,10 +845,15 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -759,43 +891,16 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="17" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1114,43 +1219,43 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DE0EC2B-16AC-4837-9A90-74B674A1A8AC}">
-  <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.5703125" customWidth="1"/>
-    <col min="2" max="2" width="28.28515625" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" customWidth="1"/>
-    <col min="4" max="4" width="32.28515625" customWidth="1"/>
-    <col min="5" max="5" width="27.7109375" customWidth="1"/>
-    <col min="6" max="6" width="49.140625" customWidth="1"/>
-    <col min="7" max="7" width="37.7109375" customWidth="1"/>
-    <col min="9" max="9" width="13.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="6.54296875" customWidth="1"/>
+    <col min="2" max="2" width="28.26953125" customWidth="1"/>
+    <col min="3" max="3" width="26.54296875" customWidth="1"/>
+    <col min="4" max="4" width="32.26953125" customWidth="1"/>
+    <col min="5" max="5" width="27.7265625" customWidth="1"/>
+    <col min="6" max="6" width="49.1796875" customWidth="1"/>
+    <col min="7" max="7" width="37.7265625" customWidth="1"/>
+    <col min="9" max="9" width="13.1796875" customWidth="1"/>
+    <col min="10" max="10" width="18.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A1" s="34"/>
-      <c r="B1" s="35"/>
-      <c r="C1" s="32" t="s">
+    <row r="1" spans="1:10" ht="31" x14ac:dyDescent="0.7">
+      <c r="A1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-    </row>
-    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+    </row>
+    <row r="2" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="45" t="s">
+      <c r="B2" s="49"/>
+      <c r="C2" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="45"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="11"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1158,11 +1263,11 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+    <row r="3" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="41"/>
+      <c r="B3" s="51"/>
       <c r="C3" s="19" t="s">
         <v>14</v>
       </c>
@@ -1174,15 +1279,15 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+    <row r="4" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="48" t="s">
+      <c r="B4" s="53"/>
+      <c r="C4" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="49"/>
+      <c r="D4" s="22"/>
       <c r="E4" s="11"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -1190,29 +1295,29 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="44"/>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="44"/>
-      <c r="H5" s="44"/>
-      <c r="I5" s="44"/>
-      <c r="J5" s="44"/>
-    </row>
-    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="54"/>
+      <c r="B5" s="54"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+    </row>
+    <row r="6" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="51"/>
+      <c r="D6" s="24"/>
       <c r="E6" s="12" t="s">
         <v>6</v>
       </c>
@@ -1225,36 +1330,36 @@
       <c r="H6" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="36" t="s">
+      <c r="I6" s="46" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="37"/>
-    </row>
-    <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="J6" s="47"/>
+    </row>
+    <row r="7" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="7"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="28"/>
-    </row>
-    <row r="8" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="37"/>
+    </row>
+    <row r="8" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="47"/>
+      <c r="D8" s="26"/>
       <c r="E8" s="18"/>
       <c r="F8" s="16" t="s">
         <v>22</v>
@@ -1265,20 +1370,20 @@
       <c r="H8" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="I8" s="52"/>
-      <c r="J8" s="24"/>
-    </row>
-    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="I8" s="57"/>
+      <c r="J8" s="35"/>
+    </row>
+    <row r="9" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="47"/>
+      <c r="D9" s="26"/>
       <c r="E9" s="3"/>
       <c r="F9" s="16" t="s">
         <v>27</v>
@@ -1289,20 +1394,20 @@
       <c r="H9" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="23"/>
-      <c r="J9" s="24"/>
-    </row>
-    <row r="10" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="I9" s="34"/>
+      <c r="J9" s="35"/>
+    </row>
+    <row r="10" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="47"/>
+      <c r="D10" s="26"/>
       <c r="E10" s="3"/>
       <c r="F10" s="16" t="s">
         <v>31</v>
@@ -1316,17 +1421,17 @@
       <c r="I10" s="4"/>
       <c r="J10" s="5"/>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="54"/>
+      <c r="D11" s="39"/>
       <c r="E11" s="3"/>
       <c r="F11" s="16" t="s">
         <v>35</v>
@@ -1340,17 +1445,17 @@
       <c r="I11" s="4"/>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="47"/>
+      <c r="D12" s="26"/>
       <c r="E12" s="3"/>
       <c r="F12" s="16" t="s">
         <v>39</v>
@@ -1364,23 +1469,23 @@
       <c r="I12" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="J12" s="24"/>
-    </row>
-    <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J12" s="35"/>
+    </row>
+    <row r="13" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="13" t="s">
         <v>16</v>
       </c>
       <c r="B13" s="14"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="28"/>
-    </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="37"/>
+    </row>
+    <row r="14" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>1</v>
       </c>
@@ -1401,12 +1506,12 @@
       <c r="H14" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="I14" s="23" t="s">
+      <c r="I14" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="24"/>
-    </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="J14" s="35"/>
+    </row>
+    <row r="15" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>2</v>
       </c>
@@ -1416,7 +1521,7 @@
       <c r="C15" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="22"/>
+      <c r="D15" s="32"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3" t="s">
         <v>49</v>
@@ -1427,20 +1532,20 @@
       <c r="H15" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="I15" s="23"/>
-      <c r="J15" s="24"/>
-    </row>
-    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="I15" s="34"/>
+      <c r="J15" s="35"/>
+    </row>
+    <row r="16" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>3</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="22"/>
+      <c r="D16" s="32"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3" t="s">
         <v>53</v>
@@ -1451,22 +1556,22 @@
       <c r="H16" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="I16" s="23" t="s">
+      <c r="I16" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="J16" s="24"/>
-    </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="J16" s="35"/>
+    </row>
+    <row r="17" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>4</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C17" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="22"/>
+      <c r="D17" s="32"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3" t="s">
         <v>57</v>
@@ -1477,26 +1582,26 @@
       <c r="H17" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="I17" s="56" t="s">
+      <c r="I17" s="40" t="s">
         <v>61</v>
       </c>
-      <c r="J17" s="57"/>
-    </row>
-    <row r="18" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="J17" s="41"/>
+    </row>
+    <row r="18" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A18" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B18" s="14"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="28"/>
-    </row>
-    <row r="19" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="36"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="36"/>
+      <c r="J18" s="37"/>
+    </row>
+    <row r="19" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>1</v>
       </c>
@@ -1507,44 +1612,44 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="17"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="24"/>
-    </row>
-    <row r="20" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="I19" s="34"/>
+      <c r="J19" s="35"/>
+    </row>
+    <row r="20" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>2</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="31"/>
-      <c r="D20" s="22"/>
+      <c r="D20" s="32"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="15"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="24"/>
-    </row>
-    <row r="21" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="I20" s="34"/>
+      <c r="J20" s="35"/>
+    </row>
+    <row r="21" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>3</v>
       </c>
       <c r="B21" s="3"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="22"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="32"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="15"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="24"/>
-    </row>
-    <row r="22" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="I21" s="34"/>
+      <c r="J21" s="35"/>
+    </row>
+    <row r="22" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>4</v>
       </c>
       <c r="B22" s="3"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="22"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="32"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -1552,214 +1657,346 @@
       <c r="I22" s="4"/>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>5</v>
       </c>
       <c r="B23" s="3"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="26"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="15"/>
-      <c r="I23" s="23"/>
-      <c r="J23" s="24"/>
-    </row>
-    <row r="24" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="I23" s="34"/>
+      <c r="J23" s="35"/>
+    </row>
+    <row r="24" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>18</v>
       </c>
       <c r="B24" s="14"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="28"/>
-    </row>
-    <row r="25" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="36"/>
+      <c r="J24" s="37"/>
+    </row>
+    <row r="25" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>1</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="29"/>
+      <c r="B25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>64</v>
+      </c>
       <c r="D25" s="30"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="23"/>
-      <c r="J25" s="24"/>
-    </row>
-    <row r="26" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="E25" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="J25" s="35"/>
+    </row>
+    <row r="26" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>2</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="22"/>
+      <c r="B26" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="D26" s="32"/>
       <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="24"/>
-    </row>
-    <row r="27" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
-        <v>3</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="24"/>
-    </row>
-    <row r="28" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="F26" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I26" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="J26" s="35"/>
+    </row>
+    <row r="27" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="14"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="36"/>
+      <c r="J27" s="37"/>
+    </row>
+    <row r="28" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B28" s="3"/>
-      <c r="C28" s="21"/>
-      <c r="D28" s="22"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="30"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="5"/>
-    </row>
-    <row r="29" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="H28" s="17"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="35"/>
+    </row>
+    <row r="29" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B29" s="3"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="26"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="32"/>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="15"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="24"/>
-    </row>
-    <row r="30" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="28"/>
-    </row>
-    <row r="31" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="I29" s="34"/>
+      <c r="J29" s="35"/>
+    </row>
+    <row r="30" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="2">
+        <v>3</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="35"/>
+    </row>
+    <row r="31" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B31" s="3"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="30"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="32"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
-      <c r="H31" s="17"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="24"/>
-    </row>
-    <row r="32" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="H31" s="15"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="5"/>
+    </row>
+    <row r="32" spans="1:10" ht="23.5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B32" s="3"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="22"/>
+      <c r="C32" s="27"/>
+      <c r="D32" s="28"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="15"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="24"/>
-    </row>
-    <row r="33" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+      <c r="I32" s="34"/>
+      <c r="J32" s="35"/>
+    </row>
+    <row r="33" spans="1:10" ht="18.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="14"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
+      <c r="E33" s="36"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="36"/>
+      <c r="J33" s="37"/>
+    </row>
+    <row r="34" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="2">
+        <v>1</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C34" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D34" s="30"/>
+      <c r="E34" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I34" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="J34" s="35"/>
+    </row>
+    <row r="35" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A35" s="2">
+        <v>2</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="D35" s="58"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I35" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="J35" s="35"/>
+    </row>
+    <row r="36" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+      <c r="A36" s="2">
         <v>3</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="24"/>
-    </row>
-    <row r="34" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+      <c r="B36" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36" s="30"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="I36" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="J36" s="35"/>
+    </row>
+    <row r="37" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A37" s="2">
         <v>4</v>
       </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="5"/>
-    </row>
-    <row r="35" spans="1:10" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+      <c r="B37" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="29" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="30"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I37" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="J37" s="35"/>
+    </row>
+    <row r="38" spans="1:10" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="2">
         <v>5</v>
       </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="26"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="15"/>
-      <c r="I35" s="23"/>
-      <c r="J35" s="24"/>
+      <c r="B38" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38" s="30"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="I38" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="J38" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="58">
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="C13:J13"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="C18:J18"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="I17:J17"/>
+  <mergeCells count="64">
+    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="C33:J33"/>
+    <mergeCell ref="C34:D34"/>
+    <mergeCell ref="I34:J34"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="I32:J32"/>
+    <mergeCell ref="C27:J27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="C24:J24"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="I26:J26"/>
     <mergeCell ref="I23:J23"/>
     <mergeCell ref="C1:J1"/>
     <mergeCell ref="A1:B1"/>
@@ -1774,26 +2011,30 @@
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I14:J14"/>
     <mergeCell ref="I16:J16"/>
-    <mergeCell ref="C24:J24"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="C30:J30"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="C34:D34"/>
-    <mergeCell ref="C35:D35"/>
-    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="C13:J13"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="C18:J18"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>